<commit_message>
fix: resolve final code review findings
</commit_message>
<xml_diff>
--- a/sample_data/pracownicy_demo.xlsx
+++ b/sample_data/pracownicy_demo.xlsx
@@ -504,12 +504,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>?ucja</t>
+          <t>Łucja</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>?urawska</t>
+          <t>Żurawska</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -551,7 +551,7 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>Specjalistka ds. jako?ci</t>
+          <t>Specjalistka ds. jakości</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
@@ -563,12 +563,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Micha?</t>
+          <t>Michał</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>G?bal</t>
+          <t>Gębal</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -592,12 +592,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>??d?</t>
+          <t>Łódź</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>?wi?tokrzyska</t>
+          <t>Świętokrzyska</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -625,7 +625,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>?wikli?ska</t>
+          <t>Ćwiklińska</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -647,12 +647,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Gda?sk</t>
+          <t>Gdańsk</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>D?uga</t>
+          <t>Długa</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">

</xml_diff>